<commit_message>
Update NPI Dashboard 2026-06-26 13:22
</commit_message>
<xml_diff>
--- a/MP变动记录.xlsx
+++ b/MP变动记录.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K311"/>
+  <dimension ref="A1:K315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16778,27 +16778,27 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>26VL</t>
+          <t>265L</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Modern A16 LE J1M</t>
+          <t>Crosshair A16 HX MLG Edition E8WEK</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>RMB 100 35W</t>
+          <t>DRG-HX 55W</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>杜晨光</t>
+          <t>朱欣怡</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -16808,52 +16808,52 @@
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>2026/06/25</t>
+          <t>2026/07/08</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>2026/07/08</t>
+          <t>2026/07/10</t>
         </is>
       </c>
       <c r="I299" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>1)物料 WLAN：5/28 ETA* 10K ,   Adapter ：目標6K， 需pull-in到06/15  ETA 2)認證  CE 06/06 ready ，PH  NTC 認證：需reddot 客戶協助CE Ready+3W 拿證，預計6/E 只能滿足PH地區出貨，EU：TUV 認證预计7/E ，其他地區認證follow  In house 流程，有訂單需求後由業務通知申請 3)TYPEC+USB4接口 SI测试Fail，需主板升级，微步確認評估預計最快7/8 TTM，已同步請微步内部評估和供应商沟通，按6月底的目标推进，待微步確認回復，Schedule TBD</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>2026/05/28 14:07:11</t>
+          <t>2026/06/26 13:22:28</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>26VL</t>
+          <t>265L</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Modern A16 LE J1M</t>
+          <t>Crosshair A16 HX MLG Edition E8WFK</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>RMB 100 35W</t>
+          <t>DRG-HX 55W</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>杜晨光</t>
+          <t>朱欣怡</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -16863,52 +16863,52 @@
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t>2026/06/25</t>
+          <t>2026/07/08</t>
         </is>
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>2026/07/08</t>
+          <t>2026/07/10</t>
         </is>
       </c>
       <c r="I300" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="J300" t="inlineStr">
         <is>
-          <t>1)物料 WLAN：5/28 ETA* 10K ,   Adapter ：目標6K， 需pull-in到06/15  ETA 2)認證  CE 06/06 ready ，PH  NTC 認證：需reddot 客戶協助CE Ready+3W 拿證，預計6/E 只能滿足PH地區出貨，EU：TUV 認證预计7/E ，其他地區認證follow  In house 流程，有訂單需求後由業務通知申請 3)TYPEC+USB4接口 SI测试Fail，需主板升级，微步確認評估預計最快7/8 TTM，已同步請微步内部評估和供应商沟通，按6月底的目标推进，待微步確認回復，Schedule TBD</t>
+          <t>1) 認證：SRRC認證中, 影響中國區出貨（可清關出貨，但上架售賣有風險）需在7/8前完成；2) Packing: WW版本設計確認中;3) Schedule: 生管排程, ATS 由7/1更新為7/3. MP @7/10</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
         <is>
-          <t>2026/05/28 14:17:44</t>
+          <t>2026/06/26 13:22:28</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>26VL</t>
+          <t>265L</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Modern A16 LE J1M</t>
+          <t>Crosshair A16 HX MLG Edition E8WGK</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>RMB 100 35W</t>
+          <t>DRG-HX 55W</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>杜晨光</t>
+          <t>朱欣怡</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -16918,25 +16918,25 @@
       </c>
       <c r="G301" t="inlineStr">
         <is>
-          <t>2026/06/25</t>
+          <t>2026/07/08</t>
         </is>
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>2026/07/08</t>
+          <t>2026/07/10</t>
         </is>
       </c>
       <c r="I301" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>1)物料 WLAN：5/28 ETA* 10K ,   Adapter ：目標6K， 需pull-in到06/15  ETA 2)認證  CE 06/06 ready ，PH  NTC 認證：需reddot 客戶協助CE Ready+3W 拿證，預計6/E 只能滿足PH地區出貨，EU：TUV 認證预计7/E ，其他地區認證follow  In house 流程，有訂單需求後由業務通知申請 3)TYPEC+USB4接口 SI测试Fail，需主板升级，微步確認評估預計最快7/8 TTM，已同步請微步内部評估和供应商沟通，按6月底的目标推进，待微步確認回復，Schedule TBD</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
         <is>
-          <t>2026/05/28 14:27:19</t>
+          <t>2026/06/26 13:22:28</t>
         </is>
       </c>
     </row>
@@ -16991,7 +16991,7 @@
       </c>
       <c r="K302" t="inlineStr">
         <is>
-          <t>2026/05/28 14:42:30</t>
+          <t>2026/05/28 14:07:11</t>
         </is>
       </c>
     </row>
@@ -17046,7 +17046,7 @@
       </c>
       <c r="K303" t="inlineStr">
         <is>
-          <t>2026/05/28 14:54:18</t>
+          <t>2026/05/28 14:17:44</t>
         </is>
       </c>
     </row>
@@ -17101,7 +17101,7 @@
       </c>
       <c r="K304" t="inlineStr">
         <is>
-          <t>2026/05/28 15:00:33</t>
+          <t>2026/05/28 14:27:19</t>
         </is>
       </c>
     </row>
@@ -17156,7 +17156,7 @@
       </c>
       <c r="K305" t="inlineStr">
         <is>
-          <t>2026/05/28 15:12:31</t>
+          <t>2026/05/28 14:42:30</t>
         </is>
       </c>
     </row>
@@ -17211,7 +17211,7 @@
       </c>
       <c r="K306" t="inlineStr">
         <is>
-          <t>2026/05/28 15:22:48</t>
+          <t>2026/05/28 14:54:18</t>
         </is>
       </c>
     </row>
@@ -17266,7 +17266,7 @@
       </c>
       <c r="K307" t="inlineStr">
         <is>
-          <t>2026/05/28 15:30:50</t>
+          <t>2026/05/28 15:00:33</t>
         </is>
       </c>
     </row>
@@ -17321,7 +17321,7 @@
       </c>
       <c r="K308" t="inlineStr">
         <is>
-          <t>2026/05/28 15:36:04</t>
+          <t>2026/05/28 15:12:31</t>
         </is>
       </c>
     </row>
@@ -17371,12 +17371,12 @@
       </c>
       <c r="J309" t="inlineStr">
         <is>
-          <t>1)物料： adapter：目標6K， 2.8K ETA @ 6/15,其它7/B 陸續進料 B&amp;S物料：6/9 釋放PO給微步，需要微步6/12協助下單備料，目前規劃ATS 6/20 SMT，物料需在6/18前寄送到微步 2)認證   a)CE：預計6/12認證ready  b)CB：24VL 6/2通知啟動認證，預計6/E ready  C)TUV 認證预计7/E  d)其他地區認證follow In house 流程，有訂單需求後由業務通知申請 e) 24VL/26VL只有TH&amp;SG下單， Total 2072 Pcs：26VL:1.8K TH+80Pcs SG &amp; 24VL: 192Pcs SG  ,SG 無需認證，TH 已通知業務安排申請認證流程（待業務回復） 3)TYPEC+USB4接口 SI测试Fail，需主板升级，6/8已安排SMT驗證，需微步加快SI驗證，已協調微步6/13到昆山更換PCBA， 4）MVT Issue 微步Debug 進度緩慢，需微步協調人力加速釐清Issue及導入對策，deadline 6/19</t>
+          <t>1)物料 WLAN：5/28 ETA* 10K ,   Adapter ：目標6K， 需pull-in到06/15  ETA 2)認證  CE 06/06 ready ，PH  NTC 認證：需reddot 客戶協助CE Ready+3W 拿證，預計6/E 只能滿足PH地區出貨，EU：TUV 認證预计7/E ，其他地區認證follow  In house 流程，有訂單需求後由業務通知申請 3)TYPEC+USB4接口 SI测试Fail，需主板升级，微步確認評估預計最快7/8 TTM，已同步請微步内部評估和供应商沟通，按6月底的目标推进，待微步確認回復，Schedule TBD</t>
         </is>
       </c>
       <c r="K309" t="inlineStr">
         <is>
-          <t>2026/06/15 13:44:06</t>
+          <t>2026/05/28 15:22:48</t>
         </is>
       </c>
     </row>
@@ -17426,12 +17426,12 @@
       </c>
       <c r="J310" t="inlineStr">
         <is>
-          <t>1)物料： adapter：目標6K， 2.8K ETA @ 6/15,其它7/B 陸續進料 B&amp;S物料：6/9 釋放PO給微步，需要微步6/12協助下單備料，目前規劃ATS 6/20 SMT，物料需在6/18前寄送到微步 2)認證   a)CE：預計6/12認證ready  b)CB：24VL 6/2通知啟動認證，預計6/E ready  C)TUV 認證预计7/E  d)其他地區認證follow In house 流程，有訂單需求後由業務通知申請 e) 24VL/26VL只有TH&amp;SG下單， Total 2072 Pcs：26VL:1.8K TH+80Pcs SG &amp; 24VL: 192Pcs SG  ,SG 無需認證，TH 已通知業務安排申請認證流程（待業務回復） 3)TYPEC+USB4接口 SI测试Fail，需主板升级，6/8已安排SMT驗證，需微步加快SI驗證，已協調微步6/13到昆山更換PCBA， 4）MVT Issue 微步Debug 進度緩慢，需微步協調人力加速釐清Issue及導入對策，deadline 6/19</t>
+          <t>1)物料 WLAN：5/28 ETA* 10K ,   Adapter ：目標6K， 需pull-in到06/15  ETA 2)認證  CE 06/06 ready ，PH  NTC 認證：需reddot 客戶協助CE Ready+3W 拿證，預計6/E 只能滿足PH地區出貨，EU：TUV 認證预计7/E ，其他地區認證follow  In house 流程，有訂單需求後由業務通知申請 3)TYPEC+USB4接口 SI测试Fail，需主板升级，微步確認評估預計最快7/8 TTM，已同步請微步内部評估和供应商沟通，按6月底的目标推进，待微步確認回復，Schedule TBD</t>
         </is>
       </c>
       <c r="K310" t="inlineStr">
         <is>
-          <t>2026/06/15 13:47:47</t>
+          <t>2026/05/28 15:30:50</t>
         </is>
       </c>
     </row>
@@ -17481,12 +17481,232 @@
       </c>
       <c r="J311" t="inlineStr">
         <is>
+          <t>1)物料 WLAN：5/28 ETA* 10K ,   Adapter ：目標6K， 需pull-in到06/15  ETA 2)認證  CE 06/06 ready ，PH  NTC 認證：需reddot 客戶協助CE Ready+3W 拿證，預計6/E 只能滿足PH地區出貨，EU：TUV 認證预计7/E ，其他地區認證follow  In house 流程，有訂單需求後由業務通知申請 3)TYPEC+USB4接口 SI测试Fail，需主板升级，微步確認評估預計最快7/8 TTM，已同步請微步内部評估和供应商沟通，按6月底的目标推进，待微步確認回復，Schedule TBD</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>2026/05/28 15:36:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>26VL</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Modern A16 LE J1M</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>RMB 100 35W</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>杜晨光</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>2026/06/25</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>2026/07/08</t>
+        </is>
+      </c>
+      <c r="I312" t="n">
+        <v>13</v>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
           <t>1)物料： adapter：目標6K， 2.8K ETA @ 6/15,其它7/B 陸續進料 B&amp;S物料：6/9 釋放PO給微步，需要微步6/12協助下單備料，目前規劃ATS 6/20 SMT，物料需在6/18前寄送到微步 2)認證   a)CE：預計6/12認證ready  b)CB：24VL 6/2通知啟動認證，預計6/E ready  C)TUV 認證预计7/E  d)其他地區認證follow In house 流程，有訂單需求後由業務通知申請 e) 24VL/26VL只有TH&amp;SG下單， Total 2072 Pcs：26VL:1.8K TH+80Pcs SG &amp; 24VL: 192Pcs SG  ,SG 無需認證，TH 已通知業務安排申請認證流程（待業務回復） 3)TYPEC+USB4接口 SI测试Fail，需主板升级，6/8已安排SMT驗證，需微步加快SI驗證，已協調微步6/13到昆山更換PCBA， 4）MVT Issue 微步Debug 進度緩慢，需微步協調人力加速釐清Issue及導入對策，deadline 6/19</t>
         </is>
       </c>
-      <c r="K311" t="inlineStr">
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>2026/06/15 13:44:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>26VL</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Modern A16 LE J1M</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>RMB 100 35W</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>杜晨光</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>2026/06/25</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>2026/07/08</t>
+        </is>
+      </c>
+      <c r="I313" t="n">
+        <v>13</v>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>1)物料： adapter：目標6K， 2.8K ETA @ 6/15,其它7/B 陸續進料 B&amp;S物料：6/9 釋放PO給微步，需要微步6/12協助下單備料，目前規劃ATS 6/20 SMT，物料需在6/18前寄送到微步 2)認證   a)CE：預計6/12認證ready  b)CB：24VL 6/2通知啟動認證，預計6/E ready  C)TUV 認證预计7/E  d)其他地區認證follow In house 流程，有訂單需求後由業務通知申請 e) 24VL/26VL只有TH&amp;SG下單， Total 2072 Pcs：26VL:1.8K TH+80Pcs SG &amp; 24VL: 192Pcs SG  ,SG 無需認證，TH 已通知業務安排申請認證流程（待業務回復） 3)TYPEC+USB4接口 SI测试Fail，需主板升级，6/8已安排SMT驗證，需微步加快SI驗證，已協調微步6/13到昆山更換PCBA， 4）MVT Issue 微步Debug 進度緩慢，需微步協調人力加速釐清Issue及導入對策，deadline 6/19</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>2026/06/15 13:47:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>26VL</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Modern A16 LE J1M</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>RMB 100 35W</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>杜晨光</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>2026/06/25</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>2026/07/08</t>
+        </is>
+      </c>
+      <c r="I314" t="n">
+        <v>13</v>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>1)物料： adapter：目標6K， 2.8K ETA @ 6/15,其它7/B 陸續進料 B&amp;S物料：6/9 釋放PO給微步，需要微步6/12協助下單備料，目前規劃ATS 6/20 SMT，物料需在6/18前寄送到微步 2)認證   a)CE：預計6/12認證ready  b)CB：24VL 6/2通知啟動認證，預計6/E ready  C)TUV 認證预计7/E  d)其他地區認證follow In house 流程，有訂單需求後由業務通知申請 e) 24VL/26VL只有TH&amp;SG下單， Total 2072 Pcs：26VL:1.8K TH+80Pcs SG &amp; 24VL: 192Pcs SG  ,SG 無需認證，TH 已通知業務安排申請認證流程（待業務回復） 3)TYPEC+USB4接口 SI测试Fail，需主板升级，6/8已安排SMT驗證，需微步加快SI驗證，已協調微步6/13到昆山更換PCBA， 4）MVT Issue 微步Debug 進度緩慢，需微步協調人力加速釐清Issue及導入對策，deadline 6/19</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
         <is>
           <t>2026/06/15 13:49:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>26VL</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Modern A16 LE J1M</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>RMB 100 35W</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>杜晨光</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>2026/07/08</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>2026/07/13</t>
+        </is>
+      </c>
+      <c r="I315" t="n">
+        <v>5</v>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>1)	Schedule：MVT Issue，需微步協調人力加速，確保在6/29前釐清Issue及導入對策，AMD  VGA WHQL  driver需在6/26 提供，滿足7/3 ATS start,</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>2026/06/26 13:22:28</t>
         </is>
       </c>
     </row>

</xml_diff>